<commit_message>
chore: reorganize repo and harden KPI upload pipeline
Archive one-off scripts, add agent skills and workflow docs, refresh
production position reference, and extend converter identity validation
with 115 passing regression tests.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/outputs/019ede9f-kpi-impact-production/KPI_Upload_Production_HO_Missing_Impact_20260619_SNAPSHOT.xlsx
+++ b/outputs/019ede9f-kpi-impact-production/KPI_Upload_Production_HO_Missing_Impact_20260619_SNAPSHOT.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Template" sheetId="1" r:id="R7ca00d97cef5434b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI Template" sheetId="1" r:id="R53e46f786d304330"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -390,7 +390,9 @@
       <x:c r="B2" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C2" s="9" t="str"/>
+      <x:c r="C2" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D2" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -443,7 +445,9 @@
       <x:c r="B3" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C3" s="9" t="str"/>
+      <x:c r="C3" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D3" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -499,7 +503,9 @@
       <x:c r="B4" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C4" s="9" t="str"/>
+      <x:c r="C4" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D4" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -551,7 +557,9 @@
       <x:c r="B5" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C5" s="9" t="str"/>
+      <x:c r="C5" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D5" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -603,7 +611,9 @@
       <x:c r="B6" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C6" s="9" t="str"/>
+      <x:c r="C6" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D6" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -655,7 +665,9 @@
       <x:c r="B7" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C7" s="9" t="str"/>
+      <x:c r="C7" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D7" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -707,7 +719,9 @@
       <x:c r="B8" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="str"/>
+      <x:c r="C8" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D8" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -759,7 +773,9 @@
       <x:c r="B9" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C9" s="9" t="str"/>
+      <x:c r="C9" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -811,7 +827,9 @@
       <x:c r="B10" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C10" s="9" t="str"/>
+      <x:c r="C10" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -866,7 +884,9 @@
       <x:c r="B11" s="9" t="str">
         <x:v>Department Hubungan Lembaga dan Investor</x:v>
       </x:c>
-      <x:c r="C11" s="9" t="str"/>
+      <x:c r="C11" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D11" s="9" t="str">
         <x:v>Department Head Hubungan Lembaga dan Investor</x:v>
       </x:c>
@@ -918,7 +938,9 @@
       <x:c r="B12" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C12" s="9" t="str"/>
+      <x:c r="C12" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -971,7 +993,9 @@
       <x:c r="B13" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C13" s="9" t="str"/>
+      <x:c r="C13" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1027,7 +1051,9 @@
       <x:c r="B14" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C14" s="9" t="str"/>
+      <x:c r="C14" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D14" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1079,7 +1105,9 @@
       <x:c r="B15" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C15" s="9" t="str"/>
+      <x:c r="C15" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D15" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1131,7 +1159,9 @@
       <x:c r="B16" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C16" s="9" t="str"/>
+      <x:c r="C16" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D16" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1183,7 +1213,9 @@
       <x:c r="B17" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C17" s="9" t="str"/>
+      <x:c r="C17" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D17" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1235,7 +1267,9 @@
       <x:c r="B18" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C18" s="9" t="str"/>
+      <x:c r="C18" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D18" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1287,7 +1321,9 @@
       <x:c r="B19" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C19" s="9" t="str"/>
+      <x:c r="C19" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D19" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1339,7 +1375,9 @@
       <x:c r="B20" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C20" s="9" t="str"/>
+      <x:c r="C20" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D20" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1394,7 +1432,9 @@
       <x:c r="B21" s="9" t="str">
         <x:v>Department Manajemen Kearsipan dan HRIS</x:v>
       </x:c>
-      <x:c r="C21" s="9" t="str"/>
+      <x:c r="C21" s="9" t="str">
+        <x:v>DIREKTORAT SDM &amp; UMUM</x:v>
+      </x:c>
       <x:c r="D21" s="9" t="str">
         <x:v>Department Head Manajemen Kearsipan, HRIS dan Administrasi SDM</x:v>
       </x:c>
@@ -1974,7 +2014,9 @@
       <x:c r="B32" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C32" s="9" t="str"/>
+      <x:c r="C32" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D32" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2027,7 +2069,9 @@
       <x:c r="B33" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C33" s="9" t="str"/>
+      <x:c r="C33" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D33" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2083,7 +2127,9 @@
       <x:c r="B34" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C34" s="9" t="str"/>
+      <x:c r="C34" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D34" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2135,7 +2181,9 @@
       <x:c r="B35" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C35" s="9" t="str"/>
+      <x:c r="C35" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D35" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2187,7 +2235,9 @@
       <x:c r="B36" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C36" s="9" t="str"/>
+      <x:c r="C36" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D36" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2239,7 +2289,9 @@
       <x:c r="B37" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C37" s="9" t="str"/>
+      <x:c r="C37" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D37" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2291,7 +2343,9 @@
       <x:c r="B38" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C38" s="9" t="str"/>
+      <x:c r="C38" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D38" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2343,7 +2397,9 @@
       <x:c r="B39" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C39" s="9" t="str"/>
+      <x:c r="C39" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D39" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2395,7 +2451,9 @@
       <x:c r="B40" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C40" s="9" t="str"/>
+      <x:c r="C40" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D40" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -2450,7 +2508,9 @@
       <x:c r="B41" s="9" t="str">
         <x:v>Department Riset dan Inovasi</x:v>
       </x:c>
-      <x:c r="C41" s="9" t="str"/>
+      <x:c r="C41" s="9" t="str">
+        <x:v>DIREKTORAT UTAMA</x:v>
+      </x:c>
       <x:c r="D41" s="9" t="str">
         <x:v>Department Head Riset dan Inovasi</x:v>
       </x:c>
@@ -42012,7 +42072,7 @@
         <x:v>781</x:v>
       </x:c>
       <x:c r="B782" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C782" s="9" t="str"/>
       <x:c r="D782" s="9" t="str">
@@ -42056,7 +42116,7 @@
       <x:c r="U782" s="9"/>
       <x:c r="V782" s="9"/>
       <x:c r="W782" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X782" s="9"/>
     </x:row>
@@ -42065,7 +42125,7 @@
         <x:v>782</x:v>
       </x:c>
       <x:c r="B783" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C783" s="9" t="str"/>
       <x:c r="D783" s="9" t="str">
@@ -42112,7 +42172,7 @@
       <x:c r="U783" s="9"/>
       <x:c r="V783" s="9"/>
       <x:c r="W783" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X783" s="9"/>
     </x:row>
@@ -42121,7 +42181,7 @@
         <x:v>783</x:v>
       </x:c>
       <x:c r="B784" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C784" s="9" t="str"/>
       <x:c r="D784" s="9" t="str">
@@ -42164,7 +42224,7 @@
       <x:c r="U784" s="9"/>
       <x:c r="V784" s="9"/>
       <x:c r="W784" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X784" s="9"/>
     </x:row>
@@ -42173,7 +42233,7 @@
         <x:v>784</x:v>
       </x:c>
       <x:c r="B785" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C785" s="9" t="str"/>
       <x:c r="D785" s="9" t="str">
@@ -42216,7 +42276,7 @@
       <x:c r="U785" s="9"/>
       <x:c r="V785" s="9"/>
       <x:c r="W785" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X785" s="9"/>
     </x:row>
@@ -42225,7 +42285,7 @@
         <x:v>785</x:v>
       </x:c>
       <x:c r="B786" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C786" s="9" t="str"/>
       <x:c r="D786" s="9" t="str">
@@ -42268,7 +42328,7 @@
       <x:c r="U786" s="9"/>
       <x:c r="V786" s="9"/>
       <x:c r="W786" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X786" s="9"/>
     </x:row>
@@ -42277,7 +42337,7 @@
         <x:v>786</x:v>
       </x:c>
       <x:c r="B787" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C787" s="9" t="str"/>
       <x:c r="D787" s="9" t="str">
@@ -42320,7 +42380,7 @@
       <x:c r="U787" s="9"/>
       <x:c r="V787" s="9"/>
       <x:c r="W787" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X787" s="9"/>
     </x:row>
@@ -42329,7 +42389,7 @@
         <x:v>787</x:v>
       </x:c>
       <x:c r="B788" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C788" s="9" t="str"/>
       <x:c r="D788" s="9" t="str">
@@ -42372,7 +42432,7 @@
       <x:c r="U788" s="9"/>
       <x:c r="V788" s="9"/>
       <x:c r="W788" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X788" s="9"/>
     </x:row>
@@ -42381,7 +42441,7 @@
         <x:v>788</x:v>
       </x:c>
       <x:c r="B789" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C789" s="9" t="str"/>
       <x:c r="D789" s="9" t="str">
@@ -42424,7 +42484,7 @@
       <x:c r="U789" s="9"/>
       <x:c r="V789" s="9"/>
       <x:c r="W789" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X789" s="9"/>
     </x:row>
@@ -42433,7 +42493,7 @@
         <x:v>789</x:v>
       </x:c>
       <x:c r="B790" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C790" s="9" t="str"/>
       <x:c r="D790" s="9" t="str">
@@ -42479,7 +42539,7 @@
       <x:c r="U790" s="9"/>
       <x:c r="V790" s="9"/>
       <x:c r="W790" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X790" s="9"/>
     </x:row>
@@ -42488,7 +42548,7 @@
         <x:v>790</x:v>
       </x:c>
       <x:c r="B791" s="9" t="str">
-        <x:v>Department Monitoring dan Evaluasi Klaster Ekspansi Korporasi</x:v>
+        <x:v>Department  Monitoring &amp; Evaluasi Klaster Ekspansi Korporasi</x:v>
       </x:c>
       <x:c r="C791" s="9" t="str"/>
       <x:c r="D791" s="9" t="str">
@@ -42531,7 +42591,7 @@
       <x:c r="U791" s="9"/>
       <x:c r="V791" s="9"/>
       <x:c r="W791" s="10" t="n">
-        <x:v>11435</x:v>
+        <x:v>11542</x:v>
       </x:c>
       <x:c r="X791" s="9"/>
     </x:row>

</xml_diff>